<commit_message>
chore: publish notes IG 1.0.0
</commit_message>
<xml_diff>
--- a/ig/notes/StructureDefinition-medcom-notes-bundle.xlsx
+++ b/ig/notes/StructureDefinition-medcom-notes-bundle.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.0-trial-use</t>
+    <t>1.0.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-10T13:54:36+00:00</t>
+    <t>2026-05-13T11:53:00+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
chore: publish notes IG 1.0.0 (#78)
Co-authored-by: tmsMedcom <tmsMedcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ig/notes/StructureDefinition-medcom-notes-bundle.xlsx
+++ b/ig/notes/StructureDefinition-medcom-notes-bundle.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.0-trial-use</t>
+    <t>1.0.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-10T13:54:36+00:00</t>
+    <t>2026-05-13T11:53:00+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>